<commit_message>
Use CLIMATH(m) as the TF core textbook in the schedule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017o9ieDcw3K8ubRqruGrPo7
</commit_message>
<xml_diff>
--- a/TF반_진도계획표_2026겨울.xlsx
+++ b/TF반_진도계획표_2026겨울.xlsx
@@ -388,7 +388,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Basecamp </t>
+      <t xml:space="preserve">CLIMATH(m) </t>
     </r>
     <r>
       <rPr>
@@ -910,7 +910,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(Basecamp)</t>
+      <t xml:space="preserve">(CLIMATH(m))</t>
     </r>
   </si>
   <si>
@@ -974,7 +974,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(Basecamp)</t>
+      <t xml:space="preserve">(CLIMATH(m))</t>
     </r>
   </si>
   <si>
@@ -1008,7 +1008,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Basecamp(</t>
+      <t xml:space="preserve">CLIMATH(m)(</t>
     </r>
     <r>
       <rPr>
@@ -1901,7 +1901,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">· Basecamp · </t>
+      <t xml:space="preserve">· CLIMATH(m) · </t>
     </r>
     <r>
       <rPr>
@@ -4518,7 +4518,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">, Basecamp) · </t>
+      <t xml:space="preserve">, CLIMATH(m)) · </t>
     </r>
     <r>
       <rPr>
@@ -4664,7 +4664,7 @@
     <t xml:space="preserve">개념</t>
   </si>
   <si>
-    <t xml:space="preserve">Basecamp</t>
+    <t xml:space="preserve">CLIMATH(m)</t>
   </si>
   <si>
     <r>

</xml_diff>